<commit_message>
Auto commit - 04301742
</commit_message>
<xml_diff>
--- a/IM/202604_Service_Count_Report.xlsx
+++ b/IM/202604_Service_Count_Report.xlsx
@@ -1311,6 +1311,9 @@
 將執行不備份更換硬碟</t>
   </si>
   <si>
+    <t>12:30:00</t>
+  </si>
+  <si>
     <t>14:57:00</t>
   </si>
   <si>
@@ -1318,9 +1321,6 @@
  更換Tm2 一二顆硬碟不備份還原最新母版 
 TM TCx800 S0902 42 0 
 HiPOS 最新版本 S0409 61 0 ARC DEF 5 408u 已跟店家告知回報代收會計</t>
-  </si>
-  <si>
-    <t>12:30:00</t>
   </si>
   <si>
     <t>11:26:00</t>
@@ -3500,9 +3500,6 @@
 門市人員測試操作正常</t>
   </si>
   <si>
-    <t>12:28:00</t>
-  </si>
-  <si>
     <t>THILF0D111</t>
   </si>
   <si>
@@ -3515,6 +3512,9 @@
     <t>更換T70
 換上 8138001526
 換下 8138001580</t>
+  </si>
+  <si>
+    <t>12:28:00</t>
   </si>
   <si>
     <t>14:16:00</t>
@@ -5959,7 +5959,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>2026042651</v>
+        <v>2026042652</v>
       </c>
       <c r="C30" s="3">
         <v>1</v>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="N30" s="6"/>
       <c r="O30" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P30" s="3"/>
       <c r="Q30" s="3">
@@ -6005,9 +6005,7 @@
       <c r="R30" s="3">
         <v>11713</v>
       </c>
-      <c r="S30" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
@@ -6029,7 +6027,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="7">
-        <v>2026042652</v>
+        <v>2026042651</v>
       </c>
       <c r="C31" s="7">
         <v>1</v>
@@ -6066,7 +6064,7 @@
       </c>
       <c r="N31" s="8"/>
       <c r="O31" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P31" s="7"/>
       <c r="Q31" s="7">
@@ -6075,7 +6073,9 @@
       <c r="R31" s="7">
         <v>11713</v>
       </c>
-      <c r="S31" s="7"/>
+      <c r="S31" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T31" s="7"/>
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
@@ -7917,7 +7917,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="7">
-        <v>2026042605</v>
+        <v>2026042604</v>
       </c>
       <c r="C59" s="7">
         <v>1</v>
@@ -7954,7 +7954,7 @@
       </c>
       <c r="N59" s="8"/>
       <c r="O59" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P59" s="7"/>
       <c r="Q59" s="7">
@@ -7963,7 +7963,9 @@
       <c r="R59" s="7">
         <v>27040</v>
       </c>
-      <c r="S59" s="7"/>
+      <c r="S59" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T59" s="7"/>
       <c r="U59" s="7"/>
       <c r="V59" s="7"/>
@@ -7985,7 +7987,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="3">
-        <v>2026042604</v>
+        <v>2026042605</v>
       </c>
       <c r="C60" s="3">
         <v>1</v>
@@ -8022,7 +8024,7 @@
       </c>
       <c r="N60" s="6"/>
       <c r="O60" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P60" s="3"/>
       <c r="Q60" s="3">
@@ -8031,9 +8033,7 @@
       <c r="R60" s="3">
         <v>27040</v>
       </c>
-      <c r="S60" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S60" s="3"/>
       <c r="T60" s="3"/>
       <c r="U60" s="3"/>
       <c r="V60" s="3"/>
@@ -8053,7 +8053,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="7">
-        <v>2026040556</v>
+        <v>2026040555</v>
       </c>
       <c r="C61" s="7">
         <v>1</v>
@@ -8090,14 +8090,16 @@
       </c>
       <c r="N61" s="8"/>
       <c r="O61" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P61" s="7"/>
       <c r="Q61" s="7"/>
       <c r="R61" s="7">
         <v>127085</v>
       </c>
-      <c r="S61" s="7"/>
+      <c r="S61" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T61" s="7"/>
       <c r="U61" s="7"/>
       <c r="V61" s="7"/>
@@ -8119,7 +8121,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="3">
-        <v>2026040555</v>
+        <v>2026040556</v>
       </c>
       <c r="C62" s="3">
         <v>1</v>
@@ -8156,16 +8158,14 @@
       </c>
       <c r="N62" s="6"/>
       <c r="O62" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P62" s="3"/>
       <c r="Q62" s="3"/>
       <c r="R62" s="3">
         <v>127085</v>
       </c>
-      <c r="S62" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S62" s="3"/>
       <c r="T62" s="3"/>
       <c r="U62" s="3"/>
       <c r="V62" s="3"/>
@@ -9519,7 +9519,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="7">
-        <v>2026043846</v>
+        <v>2026043781</v>
       </c>
       <c r="C83" s="7">
         <v>1</v>
@@ -9537,13 +9537,17 @@
         <v>256</v>
       </c>
       <c r="H83" s="7" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="I83" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="J83" s="7"/>
-      <c r="K83" s="7"/>
+      <c r="J83" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="K83" s="7" t="s">
+        <v>289</v>
+      </c>
       <c r="L83" s="8" t="s">
         <v>290</v>
       </c>
@@ -9554,26 +9558,22 @@
         <v>299</v>
       </c>
       <c r="O83" s="7" t="s">
-        <v>39</v>
+        <v>230</v>
       </c>
       <c r="P83" s="7"/>
       <c r="Q83" s="7"/>
       <c r="R83" s="7">
         <v>0</v>
       </c>
-      <c r="S83" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S83" s="7"/>
       <c r="T83" s="7"/>
       <c r="U83" s="7"/>
       <c r="V83" s="7"/>
       <c r="W83" s="7"/>
       <c r="X83" s="7"/>
-      <c r="Y83" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="Y83" s="7"/>
       <c r="Z83" s="8" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="AA83" s="7" t="s">
         <v>40</v>
@@ -9585,7 +9585,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="3">
-        <v>2026043781</v>
+        <v>2026043846</v>
       </c>
       <c r="C84" s="3">
         <v>1</v>
@@ -9603,17 +9603,13 @@
         <v>256</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>202</v>
+        <v>163</v>
       </c>
       <c r="I84" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="K84" s="3" t="s">
-        <v>289</v>
-      </c>
+      <c r="J84" s="3"/>
+      <c r="K84" s="3"/>
       <c r="L84" s="6" t="s">
         <v>290</v>
       </c>
@@ -9624,22 +9620,26 @@
         <v>299</v>
       </c>
       <c r="O84" s="3" t="s">
-        <v>230</v>
+        <v>39</v>
       </c>
       <c r="P84" s="3"/>
       <c r="Q84" s="3"/>
       <c r="R84" s="3">
         <v>0</v>
       </c>
-      <c r="S84" s="3"/>
+      <c r="S84" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T84" s="3"/>
       <c r="U84" s="3"/>
       <c r="V84" s="3"/>
       <c r="W84" s="3"/>
       <c r="X84" s="3"/>
-      <c r="Y84" s="3"/>
+      <c r="Y84" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="Z84" s="6" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="AA84" s="3" t="s">
         <v>40</v>
@@ -12279,10 +12279,10 @@
         <v>122</v>
       </c>
       <c r="B124" s="3">
-        <v>2026042587</v>
+        <v>2026042843</v>
       </c>
       <c r="C124" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>29</v>
@@ -12302,12 +12302,8 @@
       <c r="I124" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="J124" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="K124" s="3" t="s">
-        <v>289</v>
-      </c>
+      <c r="J124" s="3"/>
+      <c r="K124" s="3"/>
       <c r="L124" s="6" t="s">
         <v>290</v>
       </c>
@@ -12318,22 +12314,26 @@
         <v>421</v>
       </c>
       <c r="O124" s="3" t="s">
-        <v>230</v>
+        <v>39</v>
       </c>
       <c r="P124" s="3"/>
       <c r="Q124" s="3"/>
       <c r="R124" s="3">
         <v>0</v>
       </c>
-      <c r="S124" s="3"/>
+      <c r="S124" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T124" s="3"/>
       <c r="U124" s="3"/>
       <c r="V124" s="3"/>
       <c r="W124" s="3"/>
       <c r="X124" s="3"/>
-      <c r="Y124" s="3"/>
+      <c r="Y124" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="Z124" s="6" t="s">
-        <v>424</v>
+        <v>296</v>
       </c>
       <c r="AA124" s="3" t="s">
         <v>40</v>
@@ -12345,10 +12345,10 @@
         <v>123</v>
       </c>
       <c r="B125" s="7">
-        <v>2026042843</v>
+        <v>2026042587</v>
       </c>
       <c r="C125" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D125" s="7" t="s">
         <v>29</v>
@@ -12363,13 +12363,17 @@
         <v>116</v>
       </c>
       <c r="H125" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="I125" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="J125" s="7"/>
-      <c r="K125" s="7"/>
+      <c r="J125" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="K125" s="7" t="s">
+        <v>289</v>
+      </c>
       <c r="L125" s="8" t="s">
         <v>290</v>
       </c>
@@ -12380,26 +12384,22 @@
         <v>421</v>
       </c>
       <c r="O125" s="7" t="s">
-        <v>39</v>
+        <v>230</v>
       </c>
       <c r="P125" s="7"/>
       <c r="Q125" s="7"/>
       <c r="R125" s="7">
         <v>0</v>
       </c>
-      <c r="S125" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S125" s="7"/>
       <c r="T125" s="7"/>
       <c r="U125" s="7"/>
       <c r="V125" s="7"/>
       <c r="W125" s="7"/>
       <c r="X125" s="7"/>
-      <c r="Y125" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="Y125" s="7"/>
       <c r="Z125" s="8" t="s">
-        <v>296</v>
+        <v>425</v>
       </c>
       <c r="AA125" s="7" t="s">
         <v>40</v>
@@ -12970,7 +12970,7 @@
         <v>47</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="H134" s="3" t="s">
         <v>455</v>
@@ -14937,7 +14937,7 @@
         <v>161</v>
       </c>
       <c r="B163" s="7">
-        <v>2026040499</v>
+        <v>2026040498</v>
       </c>
       <c r="C163" s="7">
         <v>1</v>
@@ -14974,7 +14974,7 @@
       </c>
       <c r="N163" s="8"/>
       <c r="O163" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P163" s="7"/>
       <c r="Q163" s="7">
@@ -14983,9 +14983,13 @@
       <c r="R163" s="7">
         <v>15686</v>
       </c>
-      <c r="S163" s="7"/>
+      <c r="S163" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T163" s="7"/>
-      <c r="U163" s="7"/>
+      <c r="U163" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="V163" s="7"/>
       <c r="W163" s="7"/>
       <c r="X163" s="7"/>
@@ -15005,7 +15009,7 @@
         <v>162</v>
       </c>
       <c r="B164" s="3">
-        <v>2026040498</v>
+        <v>2026040499</v>
       </c>
       <c r="C164" s="3">
         <v>1</v>
@@ -15042,7 +15046,7 @@
       </c>
       <c r="N164" s="6"/>
       <c r="O164" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P164" s="3"/>
       <c r="Q164" s="3">
@@ -15051,13 +15055,9 @@
       <c r="R164" s="3">
         <v>15686</v>
       </c>
-      <c r="S164" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S164" s="3"/>
       <c r="T164" s="3"/>
-      <c r="U164" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="U164" s="3"/>
       <c r="V164" s="3"/>
       <c r="W164" s="3"/>
       <c r="X164" s="3"/>
@@ -15409,7 +15409,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="3">
-        <v>2026040109</v>
+        <v>2026040108</v>
       </c>
       <c r="C170" s="3">
         <v>1</v>
@@ -15427,7 +15427,7 @@
         <v>557</v>
       </c>
       <c r="H170" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="I170" s="3" t="s">
         <v>558</v>
@@ -15448,14 +15448,16 @@
         <v>560</v>
       </c>
       <c r="O170" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P170" s="3"/>
       <c r="Q170" s="3"/>
       <c r="R170" s="3">
         <v>27527</v>
       </c>
-      <c r="S170" s="3"/>
+      <c r="S170" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T170" s="3"/>
       <c r="U170" s="3"/>
       <c r="V170" s="3"/>
@@ -15477,7 +15479,7 @@
         <v>169</v>
       </c>
       <c r="B171" s="7">
-        <v>2026040108</v>
+        <v>2026040109</v>
       </c>
       <c r="C171" s="7">
         <v>1</v>
@@ -15495,7 +15497,7 @@
         <v>557</v>
       </c>
       <c r="H171" s="7" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="I171" s="7" t="s">
         <v>558</v>
@@ -15516,16 +15518,14 @@
         <v>560</v>
       </c>
       <c r="O171" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P171" s="7"/>
       <c r="Q171" s="7"/>
       <c r="R171" s="7">
         <v>27527</v>
       </c>
-      <c r="S171" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S171" s="7"/>
       <c r="T171" s="7"/>
       <c r="U171" s="7"/>
       <c r="V171" s="7"/>
@@ -15739,7 +15739,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="7">
-        <v>2026040463</v>
+        <v>2026040464</v>
       </c>
       <c r="C175" s="7">
         <v>1</v>
@@ -15778,16 +15778,14 @@
         <v>554</v>
       </c>
       <c r="O175" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P175" s="7"/>
       <c r="Q175" s="7"/>
       <c r="R175" s="7">
         <v>92786</v>
       </c>
-      <c r="S175" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S175" s="7"/>
       <c r="T175" s="7"/>
       <c r="U175" s="7"/>
       <c r="V175" s="7"/>
@@ -15805,7 +15803,7 @@
         <v>174</v>
       </c>
       <c r="B176" s="3">
-        <v>2026040464</v>
+        <v>2026040463</v>
       </c>
       <c r="C176" s="3">
         <v>1</v>
@@ -15844,14 +15842,16 @@
         <v>554</v>
       </c>
       <c r="O176" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P176" s="3"/>
       <c r="Q176" s="3"/>
       <c r="R176" s="3">
         <v>92786</v>
       </c>
-      <c r="S176" s="3"/>
+      <c r="S176" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T176" s="3"/>
       <c r="U176" s="3"/>
       <c r="V176" s="3"/>
@@ -16207,7 +16207,7 @@
         <v>180</v>
       </c>
       <c r="B182" s="3">
-        <v>2026040056</v>
+        <v>2026040057</v>
       </c>
       <c r="C182" s="3">
         <v>1</v>
@@ -16246,7 +16246,7 @@
         <v>560</v>
       </c>
       <c r="O182" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P182" s="3"/>
       <c r="Q182" s="3">
@@ -16255,9 +16255,7 @@
       <c r="R182" s="3">
         <v>361051</v>
       </c>
-      <c r="S182" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S182" s="3"/>
       <c r="T182" s="3"/>
       <c r="U182" s="3"/>
       <c r="V182" s="3"/>
@@ -16279,7 +16277,7 @@
         <v>181</v>
       </c>
       <c r="B183" s="7">
-        <v>2026040057</v>
+        <v>2026040056</v>
       </c>
       <c r="C183" s="7">
         <v>1</v>
@@ -16318,7 +16316,7 @@
         <v>560</v>
       </c>
       <c r="O183" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P183" s="7"/>
       <c r="Q183" s="7">
@@ -16327,7 +16325,9 @@
       <c r="R183" s="7">
         <v>361051</v>
       </c>
-      <c r="S183" s="7"/>
+      <c r="S183" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T183" s="7"/>
       <c r="U183" s="7"/>
       <c r="V183" s="7"/>
@@ -16419,7 +16419,7 @@
         <v>183</v>
       </c>
       <c r="B185" s="7">
-        <v>2026040537</v>
+        <v>2026040538</v>
       </c>
       <c r="C185" s="7">
         <v>1</v>
@@ -16458,7 +16458,7 @@
         <v>585</v>
       </c>
       <c r="O185" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P185" s="7"/>
       <c r="Q185" s="7">
@@ -16467,9 +16467,7 @@
       <c r="R185" s="7">
         <v>29387</v>
       </c>
-      <c r="S185" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S185" s="7"/>
       <c r="T185" s="7"/>
       <c r="U185" s="7"/>
       <c r="V185" s="7"/>
@@ -16479,15 +16477,19 @@
       <c r="Z185" s="8" t="s">
         <v>526</v>
       </c>
-      <c r="AA185" s="7"/>
-      <c r="AB185" s="7"/>
+      <c r="AA185" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB185" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="186" spans="1:28">
       <c r="A186" s="3">
         <v>184</v>
       </c>
       <c r="B186" s="3">
-        <v>2026040538</v>
+        <v>2026040537</v>
       </c>
       <c r="C186" s="3">
         <v>1</v>
@@ -16526,7 +16528,7 @@
         <v>585</v>
       </c>
       <c r="O186" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P186" s="3"/>
       <c r="Q186" s="3">
@@ -16535,7 +16537,9 @@
       <c r="R186" s="3">
         <v>29387</v>
       </c>
-      <c r="S186" s="3"/>
+      <c r="S186" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T186" s="3"/>
       <c r="U186" s="3"/>
       <c r="V186" s="3"/>
@@ -16545,9 +16549,7 @@
       <c r="Z186" s="6" t="s">
         <v>526</v>
       </c>
-      <c r="AA186" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA186" s="3"/>
       <c r="AB186" s="3"/>
     </row>
     <row r="187" spans="1:28">
@@ -18508,7 +18510,7 @@
         <v>185</v>
       </c>
       <c r="G216" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="H216" s="3" t="s">
         <v>661</v>
@@ -22921,7 +22923,7 @@
         <v>280</v>
       </c>
       <c r="B282" s="3">
-        <v>2026040916</v>
+        <v>2026040917</v>
       </c>
       <c r="C282" s="3">
         <v>1</v>
@@ -22960,7 +22962,7 @@
         <v>824</v>
       </c>
       <c r="O282" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P282" s="3"/>
       <c r="Q282" s="3">
@@ -22969,17 +22971,13 @@
       <c r="R282" s="3">
         <v>22500</v>
       </c>
-      <c r="S282" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S282" s="3"/>
       <c r="T282" s="3"/>
       <c r="U282" s="3"/>
       <c r="V282" s="3"/>
       <c r="W282" s="3"/>
       <c r="X282" s="3"/>
-      <c r="Y282" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="Y282" s="3"/>
       <c r="Z282" s="6" t="s">
         <v>801</v>
       </c>
@@ -22995,7 +22993,7 @@
         <v>281</v>
       </c>
       <c r="B283" s="7">
-        <v>2026040917</v>
+        <v>2026040916</v>
       </c>
       <c r="C283" s="7">
         <v>1</v>
@@ -23034,7 +23032,7 @@
         <v>824</v>
       </c>
       <c r="O283" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P283" s="7"/>
       <c r="Q283" s="7">
@@ -23043,13 +23041,17 @@
       <c r="R283" s="7">
         <v>22500</v>
       </c>
-      <c r="S283" s="7"/>
+      <c r="S283" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T283" s="7"/>
       <c r="U283" s="7"/>
       <c r="V283" s="7"/>
       <c r="W283" s="7"/>
       <c r="X283" s="7"/>
-      <c r="Y283" s="7"/>
+      <c r="Y283" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="Z283" s="8" t="s">
         <v>801</v>
       </c>
@@ -24317,7 +24319,7 @@
         <v>300</v>
       </c>
       <c r="B302" s="3">
-        <v>2026043305</v>
+        <v>2026043306</v>
       </c>
       <c r="C302" s="3">
         <v>1</v>
@@ -24356,16 +24358,14 @@
         <v>860</v>
       </c>
       <c r="O302" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P302" s="3"/>
       <c r="Q302" s="3"/>
       <c r="R302" s="3">
         <v>786</v>
       </c>
-      <c r="S302" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S302" s="3"/>
       <c r="T302" s="3"/>
       <c r="U302" s="3"/>
       <c r="V302" s="3"/>
@@ -24387,7 +24387,7 @@
         <v>301</v>
       </c>
       <c r="B303" s="7">
-        <v>2026043306</v>
+        <v>2026043305</v>
       </c>
       <c r="C303" s="7">
         <v>1</v>
@@ -24426,14 +24426,16 @@
         <v>860</v>
       </c>
       <c r="O303" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P303" s="7"/>
       <c r="Q303" s="7"/>
       <c r="R303" s="7">
         <v>786</v>
       </c>
-      <c r="S303" s="7"/>
+      <c r="S303" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T303" s="7"/>
       <c r="U303" s="7"/>
       <c r="V303" s="7"/>
@@ -24857,7 +24859,7 @@
         <v>308</v>
       </c>
       <c r="B310" s="3">
-        <v>2026040831</v>
+        <v>2026040832</v>
       </c>
       <c r="C310" s="3">
         <v>1</v>
@@ -24896,16 +24898,14 @@
         <v>873</v>
       </c>
       <c r="O310" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P310" s="3"/>
       <c r="Q310" s="3"/>
       <c r="R310" s="3">
         <v>86361</v>
       </c>
-      <c r="S310" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S310" s="3"/>
       <c r="T310" s="3"/>
       <c r="U310" s="3"/>
       <c r="V310" s="3"/>
@@ -24927,7 +24927,7 @@
         <v>309</v>
       </c>
       <c r="B311" s="7">
-        <v>2026040832</v>
+        <v>2026040831</v>
       </c>
       <c r="C311" s="7">
         <v>1</v>
@@ -24966,14 +24966,16 @@
         <v>873</v>
       </c>
       <c r="O311" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P311" s="7"/>
       <c r="Q311" s="7"/>
       <c r="R311" s="7">
         <v>86361</v>
       </c>
-      <c r="S311" s="7"/>
+      <c r="S311" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T311" s="7"/>
       <c r="U311" s="7"/>
       <c r="V311" s="7"/>
@@ -27109,7 +27111,7 @@
         <v>341</v>
       </c>
       <c r="B343" s="7">
-        <v>2026042895</v>
+        <v>2026042896</v>
       </c>
       <c r="C343" s="7">
         <v>1</v>
@@ -27148,16 +27150,14 @@
         <v>911</v>
       </c>
       <c r="O343" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P343" s="7"/>
       <c r="Q343" s="7"/>
       <c r="R343" s="7">
         <v>6975</v>
       </c>
-      <c r="S343" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S343" s="7"/>
       <c r="T343" s="7"/>
       <c r="U343" s="7"/>
       <c r="V343" s="7"/>
@@ -27167,15 +27167,19 @@
       <c r="Z343" s="8" t="s">
         <v>801</v>
       </c>
-      <c r="AA343" s="7"/>
-      <c r="AB343" s="7"/>
+      <c r="AA343" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB343" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="344" spans="1:28">
       <c r="A344" s="3">
         <v>342</v>
       </c>
       <c r="B344" s="3">
-        <v>2026042896</v>
+        <v>2026042895</v>
       </c>
       <c r="C344" s="3">
         <v>1</v>
@@ -27214,14 +27218,16 @@
         <v>911</v>
       </c>
       <c r="O344" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P344" s="3"/>
       <c r="Q344" s="3"/>
       <c r="R344" s="3">
         <v>6975</v>
       </c>
-      <c r="S344" s="3"/>
+      <c r="S344" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T344" s="3"/>
       <c r="U344" s="3"/>
       <c r="V344" s="3"/>
@@ -27231,9 +27237,7 @@
       <c r="Z344" s="6" t="s">
         <v>801</v>
       </c>
-      <c r="AA344" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA344" s="3"/>
       <c r="AB344" s="3"/>
     </row>
     <row r="345" spans="1:28">
@@ -27509,7 +27513,7 @@
         <v>347</v>
       </c>
       <c r="B349" s="7">
-        <v>2026043917</v>
+        <v>2026043911</v>
       </c>
       <c r="C349" s="7">
         <v>1</v>
@@ -27575,7 +27579,7 @@
         <v>348</v>
       </c>
       <c r="B350" s="3">
-        <v>2026043918</v>
+        <v>2026043912</v>
       </c>
       <c r="C350" s="3">
         <v>1</v>
@@ -27641,7 +27645,7 @@
         <v>349</v>
       </c>
       <c r="B351" s="7">
-        <v>2026043911</v>
+        <v>2026043917</v>
       </c>
       <c r="C351" s="7">
         <v>1</v>
@@ -27707,7 +27711,7 @@
         <v>350</v>
       </c>
       <c r="B352" s="3">
-        <v>2026043912</v>
+        <v>2026043918</v>
       </c>
       <c r="C352" s="3">
         <v>1</v>
@@ -30395,7 +30399,7 @@
         <v>390</v>
       </c>
       <c r="B392" s="3">
-        <v>2026041281</v>
+        <v>2026041280</v>
       </c>
       <c r="C392" s="3">
         <v>1</v>
@@ -30434,14 +30438,16 @@
         <v>931</v>
       </c>
       <c r="O392" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P392" s="3"/>
       <c r="Q392" s="3"/>
       <c r="R392" s="3">
         <v>359</v>
       </c>
-      <c r="S392" s="3"/>
+      <c r="S392" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T392" s="3"/>
       <c r="U392" s="3"/>
       <c r="V392" s="3"/>
@@ -30451,19 +30457,15 @@
       <c r="Z392" s="6" t="s">
         <v>801</v>
       </c>
-      <c r="AA392" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="AB392" s="3">
-        <v>1</v>
-      </c>
+      <c r="AA392" s="3"/>
+      <c r="AB392" s="3"/>
     </row>
     <row r="393" spans="1:28">
       <c r="A393" s="7">
         <v>391</v>
       </c>
       <c r="B393" s="7">
-        <v>2026041280</v>
+        <v>2026041281</v>
       </c>
       <c r="C393" s="7">
         <v>1</v>
@@ -30502,16 +30504,14 @@
         <v>931</v>
       </c>
       <c r="O393" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P393" s="7"/>
       <c r="Q393" s="7"/>
       <c r="R393" s="7">
         <v>359</v>
       </c>
-      <c r="S393" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S393" s="7"/>
       <c r="T393" s="7"/>
       <c r="U393" s="7"/>
       <c r="V393" s="7"/>
@@ -30521,7 +30521,9 @@
       <c r="Z393" s="8" t="s">
         <v>801</v>
       </c>
-      <c r="AA393" s="7"/>
+      <c r="AA393" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="AB393" s="7"/>
     </row>
     <row r="394" spans="1:28">
@@ -30943,7 +30945,7 @@
         <v>398</v>
       </c>
       <c r="B400" s="3">
-        <v>2026043307</v>
+        <v>2026043308</v>
       </c>
       <c r="C400" s="3">
         <v>1</v>
@@ -30982,16 +30984,14 @@
         <v>860</v>
       </c>
       <c r="O400" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P400" s="3"/>
       <c r="Q400" s="3"/>
       <c r="R400" s="3">
         <v>159550</v>
       </c>
-      <c r="S400" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S400" s="3"/>
       <c r="T400" s="3"/>
       <c r="U400" s="3"/>
       <c r="V400" s="3"/>
@@ -31013,7 +31013,7 @@
         <v>399</v>
       </c>
       <c r="B401" s="7">
-        <v>2026043308</v>
+        <v>2026043307</v>
       </c>
       <c r="C401" s="7">
         <v>1</v>
@@ -31052,14 +31052,16 @@
         <v>860</v>
       </c>
       <c r="O401" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P401" s="7"/>
       <c r="Q401" s="7"/>
       <c r="R401" s="7">
         <v>159550</v>
       </c>
-      <c r="S401" s="7"/>
+      <c r="S401" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T401" s="7"/>
       <c r="U401" s="7"/>
       <c r="V401" s="7"/>
@@ -33466,7 +33468,7 @@
         <v>1062</v>
       </c>
       <c r="G437" s="7" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="H437" s="7" t="s">
         <v>60</v>
@@ -34327,7 +34329,7 @@
         <v>448</v>
       </c>
       <c r="B450" s="3">
-        <v>2026042725</v>
+        <v>2026042726</v>
       </c>
       <c r="C450" s="3">
         <v>1</v>
@@ -34366,16 +34368,14 @@
         <v>1096</v>
       </c>
       <c r="O450" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P450" s="3"/>
       <c r="Q450" s="3"/>
       <c r="R450" s="3">
         <v>9617</v>
       </c>
-      <c r="S450" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S450" s="3"/>
       <c r="T450" s="3"/>
       <c r="U450" s="3"/>
       <c r="V450" s="3"/>
@@ -34385,15 +34385,19 @@
       <c r="Z450" s="6" t="s">
         <v>801</v>
       </c>
-      <c r="AA450" s="3"/>
-      <c r="AB450" s="3"/>
+      <c r="AA450" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB450" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="451" spans="1:28">
       <c r="A451" s="7">
         <v>449</v>
       </c>
       <c r="B451" s="7">
-        <v>2026042726</v>
+        <v>2026042725</v>
       </c>
       <c r="C451" s="7">
         <v>1</v>
@@ -34432,14 +34436,16 @@
         <v>1096</v>
       </c>
       <c r="O451" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="P451" s="7"/>
       <c r="Q451" s="7"/>
       <c r="R451" s="7">
         <v>9617</v>
       </c>
-      <c r="S451" s="7"/>
+      <c r="S451" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T451" s="7"/>
       <c r="U451" s="7"/>
       <c r="V451" s="7"/>
@@ -34449,9 +34455,7 @@
       <c r="Z451" s="8" t="s">
         <v>801</v>
       </c>
-      <c r="AA451" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA451" s="7"/>
       <c r="AB451" s="7"/>
     </row>
     <row r="452" spans="1:28">
@@ -35415,7 +35419,7 @@
         <v>464</v>
       </c>
       <c r="B466" s="3">
-        <v>2026041055</v>
+        <v>2026040568</v>
       </c>
       <c r="C466" s="3">
         <v>1</v>
@@ -35433,33 +35437,35 @@
         <v>130</v>
       </c>
       <c r="H466" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="I466" s="3" t="s">
         <v>1134</v>
       </c>
-      <c r="I466" s="3" t="s">
-        <v>1135</v>
-      </c>
-      <c r="J466" s="3"/>
-      <c r="K466" s="3"/>
+      <c r="J466" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="K466" s="3" t="s">
+        <v>289</v>
+      </c>
       <c r="L466" s="6" t="s">
         <v>290</v>
       </c>
       <c r="M466" s="6" t="s">
+        <v>1135</v>
+      </c>
+      <c r="N466" s="6" t="s">
         <v>1136</v>
       </c>
-      <c r="N466" s="6" t="s">
-        <v>1137</v>
-      </c>
       <c r="O466" s="3" t="s">
-        <v>39</v>
+        <v>230</v>
       </c>
       <c r="P466" s="3"/>
       <c r="Q466" s="3"/>
       <c r="R466" s="3">
         <v>0</v>
       </c>
-      <c r="S466" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S466" s="3"/>
       <c r="T466" s="3"/>
       <c r="U466" s="3"/>
       <c r="V466" s="3"/>
@@ -35467,7 +35473,7 @@
       <c r="X466" s="3"/>
       <c r="Y466" s="3"/>
       <c r="Z466" s="6" t="s">
-        <v>296</v>
+        <v>1137</v>
       </c>
       <c r="AA466" s="3" t="s">
         <v>40</v>
@@ -35481,7 +35487,7 @@
         <v>465</v>
       </c>
       <c r="B467" s="7">
-        <v>2026040568</v>
+        <v>2026041055</v>
       </c>
       <c r="C467" s="7">
         <v>1</v>
@@ -35499,35 +35505,33 @@
         <v>130</v>
       </c>
       <c r="H467" s="7" t="s">
-        <v>557</v>
+        <v>1138</v>
       </c>
       <c r="I467" s="7" t="s">
-        <v>1135</v>
-      </c>
-      <c r="J467" s="7" t="s">
-        <v>288</v>
-      </c>
-      <c r="K467" s="7" t="s">
-        <v>289</v>
-      </c>
+        <v>1134</v>
+      </c>
+      <c r="J467" s="7"/>
+      <c r="K467" s="7"/>
       <c r="L467" s="8" t="s">
         <v>290</v>
       </c>
       <c r="M467" s="8" t="s">
+        <v>1135</v>
+      </c>
+      <c r="N467" s="8" t="s">
         <v>1136</v>
       </c>
-      <c r="N467" s="8" t="s">
-        <v>1137</v>
-      </c>
       <c r="O467" s="7" t="s">
-        <v>230</v>
+        <v>39</v>
       </c>
       <c r="P467" s="7"/>
       <c r="Q467" s="7"/>
       <c r="R467" s="7">
         <v>0</v>
       </c>
-      <c r="S467" s="7"/>
+      <c r="S467" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T467" s="7"/>
       <c r="U467" s="7"/>
       <c r="V467" s="7"/>
@@ -35535,7 +35539,7 @@
       <c r="X467" s="7"/>
       <c r="Y467" s="7"/>
       <c r="Z467" s="8" t="s">
-        <v>1138</v>
+        <v>296</v>
       </c>
       <c r="AA467" s="7" t="s">
         <v>40</v>
@@ -35568,7 +35572,7 @@
         <v>1139</v>
       </c>
       <c r="I468" s="3" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="J468" s="3" t="s">
         <v>288</v>
@@ -35580,10 +35584,10 @@
         <v>290</v>
       </c>
       <c r="M468" s="6" t="s">
+        <v>1135</v>
+      </c>
+      <c r="N468" s="6" t="s">
         <v>1136</v>
-      </c>
-      <c r="N468" s="6" t="s">
-        <v>1137</v>
       </c>
       <c r="O468" s="3" t="s">
         <v>230</v>
@@ -35641,7 +35645,7 @@
         <v>1141</v>
       </c>
       <c r="AB469" s="9">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>